<commit_message>
update com funcao de distancia mais eficiente
</commit_message>
<xml_diff>
--- a/AHP-CRITERIOS_PESOS/AHP.xlsx
+++ b/AHP-CRITERIOS_PESOS/AHP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://timbrasil-my.sharepoint.com/personal/tblacerda_timbrasil_com_br/Documents/__Automacao_de_tarefas/HACK@TIM_2024/AHP-CRITERIOS_PESOS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://timbrasil-my.sharepoint.com/personal/tblacerda_timbrasil_com_br/Documents/__Automacao_de_tarefas/HACK@TIM_2024/__ENTREGAVEIS_GRUPO_XX_DANTIMZIG__/PYTHON/AHP-CRITERIOS_PESOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1239" documentId="11_F25DC773A252ABDACC104865295C53F25ADE58F6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39F1A22E-2F69-4CE0-8111-18E134B8752B}"/>
+  <xr:revisionPtr revIDLastSave="1241" documentId="11_F25DC773A252ABDACC104865295C53F25ADE58F6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{07D24BF9-F135-4049-922F-3DC0455809F3}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -122,7 +122,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="25">
   <si>
     <t>Matrix A</t>
   </si>
@@ -194,6 +194,9 @@
   </si>
   <si>
     <t>SITE SALVADOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -777,16 +780,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>247650</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>295275</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>228600</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>32</xdr:col>
-      <xdr:colOff>421725</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>141657</xdr:rowOff>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>469350</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>179757</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -809,8 +812,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13811250" y="0"/>
-          <a:ext cx="6879675" cy="5018457"/>
+          <a:off x="9677400" y="609600"/>
+          <a:ext cx="6879675" cy="5447082"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2268,7 +2271,7 @@
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B18" s="12" t="s">
         <v>19</v>

</xml_diff>